<commit_message>
data: stage coverage refresh 4/6
</commit_message>
<xml_diff>
--- a/diseases/d049/2010-2014.xlsx
+++ b/diseases/d049/2010-2014.xlsx
@@ -4295,28 +4295,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO25" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP25" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR25" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS25" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU25" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV25" t="inlineStr">
@@ -4596,28 +4610,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO27" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP27" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR27" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS27" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU27" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV27" t="inlineStr">
@@ -4744,28 +4772,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO28" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP28" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR28" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS28" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ28" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU28" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV28" t="inlineStr">
@@ -4892,28 +4934,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO29" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP29" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR29" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS29" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ29" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU29" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV29" t="inlineStr">
@@ -5040,28 +5096,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO30" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP30" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR30" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS30" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ30" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS30" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU30" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV30" t="inlineStr">
@@ -5188,28 +5258,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO31" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP31" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR31" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS31" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ31" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS31" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU31" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV31" t="inlineStr">
@@ -5489,28 +5573,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO33" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP33" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR33" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS33" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ33" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS33" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU33" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV33" t="inlineStr">
@@ -5637,28 +5735,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO34" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP34" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR34" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS34" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ34" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU34" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV34" t="inlineStr">
@@ -5785,28 +5897,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO35" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP35" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR35" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS35" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ35" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS35" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU35" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV35" t="inlineStr">
@@ -5933,28 +6059,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO36" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP36" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR36" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS36" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ36" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS36" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU36" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV36" t="inlineStr">
@@ -6234,28 +6374,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO38" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP38" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR38" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS38" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ38" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU38" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV38" t="inlineStr">
@@ -6382,28 +6536,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO39" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP39" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR39" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS39" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ39" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS39" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU39" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV39" t="inlineStr">
@@ -6530,28 +6698,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO40" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR40" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS40" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ40" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS40" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU40" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV40" t="inlineStr">
@@ -6678,28 +6860,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO41" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP41" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR41" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS41" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ41" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS41" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU41" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV41" t="inlineStr">
@@ -6826,28 +7022,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO42" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP42" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR42" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS42" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ42" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS42" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU42" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV42" t="inlineStr">
@@ -7127,28 +7337,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA44" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO44" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP44" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR44" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS44" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ44" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS44" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU44" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV44" t="inlineStr">
@@ -7275,28 +7499,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA45" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO45" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP45" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR45" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS45" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ45" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS45" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU45" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV45" t="inlineStr">
@@ -7423,28 +7661,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA46" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO46" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP46" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR46" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS46" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ46" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS46" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU46" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV46" t="inlineStr">
@@ -7571,28 +7823,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA47" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO47" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP47" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR47" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS47" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ47" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS47" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU47" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV47" t="inlineStr">
@@ -7872,28 +8138,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA49" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO49" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP49" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR49" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS49" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ49" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS49" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU49" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV49" t="inlineStr">
@@ -8020,28 +8300,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA50" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO50" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP50" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR50" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS50" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ50" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS50" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU50" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV50" t="inlineStr">
@@ -8168,28 +8462,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA51" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO51" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP51" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR51" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS51" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ51" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS51" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU51" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV51" t="inlineStr">
@@ -8316,28 +8624,42 @@
           <t>wpp_computed</t>
         </is>
       </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
       <c r="AO52" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
+          <t>mixed</t>
         </is>
       </c>
       <c r="AP52" t="inlineStr">
         <is>
-          <t>legacy_fallback</t>
-        </is>
-      </c>
-      <c r="AR52" t="inlineStr">
-        <is>
-          <t>legacy_identity_may_be_lossy</t>
-        </is>
-      </c>
-      <c r="AS52" t="inlineStr"/>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ52" t="inlineStr">
+        <is>
+          <t>legacy_gap_fill</t>
+        </is>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>HOLD_JP_165c828b0fb1b842ce8afd4aadf6</t>
+        </is>
+      </c>
       <c r="AT52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU52" t="inlineStr">
         <is>
-          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+          <t>The public curve is read directly from one registered source series. Registry facts replace matching periods; legacy-only periods are retained as explicit coverage gap fills.</t>
         </is>
       </c>
       <c r="AV52" t="inlineStr">

</xml_diff>